<commit_message>
adaptations for new naming convention and mapping columns
</commit_message>
<xml_diff>
--- a/mappings/contacts_mapping.xlsx
+++ b/mappings/contacts_mapping.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Accounts → res.partner'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Contacts → res.partner'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'PaymentCond → payment.term'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PaymentCond → payment.term.line'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Accounts → res.partner'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Contacts → res.partner'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'PaymentCond → payment.term'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PaymentCond → payment.term.line'!$A$1:$H$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G172"/>
+  <dimension ref="A1:H172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -502,7 +502,8 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="12.5" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -538,6 +539,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Related Model</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -573,7 +579,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Primary key. Named x_aa_exact_account_id to distinguish from x_aa_exact_contact_id (Contacts sheet). A company partner has this field populated; a person partner does not. Used for reconciliation, deduplication, and relationship resolution across all migrated tables.</t>
         </is>
@@ -610,7 +617,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Exact account code (fixed-length numeric string with leading spaces). Maps to Odoo's external reference field. Strip leading spaces during migration. Only Accounts set ref — Contacts do not.</t>
         </is>
@@ -647,7 +655,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Account name. Direct mapping. (Contacts derive name from FirstName + MiddleName + LastName instead.)</t>
         </is>
@@ -684,7 +693,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Exact search/short code. No Odoo equivalent.</t>
         </is>
@@ -721,7 +731,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Registered trade name. Odoo has no dedicated trade name field.</t>
         </is>
@@ -758,7 +769,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Exact customer status: A=None, S=Suspect, P=Prospect, C=Customer. Preserved for full fidelity. Also drives Derived customer_rank.</t>
         </is>
@@ -795,7 +807,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>A=Relation, D=Division. Preserve for reference.</t>
         </is>
@@ -832,7 +845,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Preserved as custom. Also drives Derived supplier_rank.</t>
         </is>
@@ -869,7 +883,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>No Odoo equivalent for reseller classification.</t>
         </is>
@@ -906,7 +921,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Values: 0=No, 1=Yes (unpublished), 2=Yes (published). No Odoo equivalent.</t>
         </is>
@@ -943,7 +959,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>No Odoo equivalent.</t>
         </is>
@@ -980,7 +997,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>No Odoo equivalent.</t>
         </is>
@@ -1017,7 +1035,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Whether account is allowed for sales. Odoo uses customer_rank &gt; 0 to filter customers, but that is semantic, not a permission flag.</t>
         </is>
@@ -1054,7 +1073,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Excluded from marketing mailings. Odoo has is_blacklisted but semantics differ. Preserve as custom.</t>
         </is>
@@ -1091,7 +1111,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Pilot account flag. No Odoo equivalent.</t>
         </is>
@@ -1128,7 +1149,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Eligibility for extra duty. No Odoo equivalent.</t>
         </is>
@@ -1165,7 +1187,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Whether account data has been anonymised. Shared field name with Contacts sheet — same field on res.partner, one per record.</t>
         </is>
@@ -1202,7 +1225,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>First address line → Odoo street. (Contacts use concatenated AddressStreet + Number + Suffix instead.)</t>
         </is>
@@ -1239,7 +1263,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Second address line → Odoo street2.</t>
         </is>
@@ -1276,7 +1301,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Odoo has only street + street2. Third line preserved as custom.</t>
         </is>
@@ -1313,7 +1339,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Direct mapping.</t>
         </is>
@@ -1350,7 +1377,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Direct mapping.</t>
         </is>
@@ -1379,7 +1407,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.country</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1388,6 +1416,11 @@
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>res.country</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Exact stores ISO country code (2-char). Resolve via res.country.code lookup.</t>
         </is>
@@ -1426,6 +1459,11 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field. Value derivable from country_id.name.</t>
         </is>
       </c>
@@ -1453,7 +1491,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.country.state</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1462,6 +1500,11 @@
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>res.country.state</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>State/Province code. Resolve via res.country.state.code + country_id lookup.</t>
         </is>
@@ -1500,6 +1543,11 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -1535,7 +1583,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>CRM creation source for the address. No Odoo equivalent.</t>
         </is>
@@ -1572,7 +1621,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Direct mapping.</t>
         </is>
@@ -1609,7 +1659,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Direct mapping.</t>
         </is>
@@ -1646,7 +1697,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Odoo has no phone extension field. Shared field name with Contacts sheet.</t>
         </is>
@@ -1683,7 +1735,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Odoo 18 has no fax field. Shared field name with Contacts sheet.</t>
         </is>
@@ -1720,7 +1773,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Direct mapping.</t>
         </is>
@@ -1757,7 +1811,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Direct mapping.</t>
         </is>
@@ -1794,7 +1849,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Direct mapping.</t>
         </is>
@@ -1831,7 +1887,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Sales credit limit. Also set use_partner_credit_limit=True if value &gt; 0 (see Derived).</t>
         </is>
@@ -1868,7 +1925,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Purchase credit limit. Odoo only has a single credit_limit (sales/receivables).</t>
         </is>
@@ -1897,7 +1955,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>many2one → account.payment.term</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1906,6 +1964,11 @@
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>account.payment.term</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Default sales payment term code. Resolve via x_aa_code lookup on account.payment.term (Payment Terms mapping). Exact stores a code string.</t>
         </is>
@@ -1944,6 +2007,11 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -1971,7 +2039,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>many2one → account.payment.term</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1980,6 +2048,11 @@
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>account.payment.term</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Default purchase payment term code. Same resolution as PaymentConditionSales.</t>
         </is>
@@ -2018,6 +2091,11 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -2045,7 +2123,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>many2one → product.pricelist</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2054,6 +2132,11 @@
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>product.pricelist</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Default sales price list. Requires product.pricelist migration/mapping.</t>
         </is>
@@ -2082,7 +2165,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.currency</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2091,6 +2174,11 @@
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>res.currency</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Sales currency code. Resolve via res.currency.name lookup.</t>
         </is>
@@ -2129,6 +2217,11 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -2156,7 +2249,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.currency</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2165,6 +2258,11 @@
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>res.currency</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Purchase currency code. Resolve via res.currency.name lookup.</t>
         </is>
@@ -2203,6 +2301,11 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -2238,7 +2341,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Default sales discount (fraction, e.g., 0.055 = 5.5%). Odoo handles discounts via pricelists.</t>
         </is>
@@ -2275,7 +2379,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>Default purchase discount (fraction). No Odoo equivalent on partner.</t>
         </is>
@@ -2312,7 +2417,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Default sales VAT code. Odoo uses fiscal positions instead.</t>
         </is>
@@ -2351,6 +2457,11 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -2386,7 +2497,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Default purchase VAT code. Odoo uses fiscal positions instead.</t>
         </is>
@@ -2425,6 +2537,11 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -2460,7 +2577,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>ID of alternate account to invoice. Odoo uses child contacts with type="invoice". Preserve GUID.</t>
         </is>
@@ -2499,6 +2617,11 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -2536,6 +2659,11 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -2571,7 +2699,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>Method of sending invoices (1=Paper, 2=Email, 4=Mailbox, 8=Send/track, 32=Peppol). Odoo has invoice_sending_method but value sets don't align.</t>
         </is>
@@ -2608,7 +2737,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>Which attachment types to send with invoices. No Odoo equivalent.</t>
         </is>
@@ -2645,7 +2775,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>Payment link active for sales. No direct Odoo partner-level equivalent.</t>
         </is>
@@ -2682,7 +2813,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>0=combined, 1=separate invoices per subscription. No Odoo equivalent on partner.</t>
         </is>
@@ -2719,7 +2851,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>Separate invoice per project. No Odoo equivalent on partner.</t>
         </is>
@@ -2756,7 +2889,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>T&amp;B consolidation scenario (0-6). No Odoo equivalent.</t>
         </is>
@@ -2793,7 +2927,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>Display remarks on sales orders. Odoo has sale_warn but works differently.</t>
         </is>
@@ -2830,7 +2965,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr"/>
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>Delivery handling (0=Partial, 1=Complete, 2=Partial without backorder). Odoo handles at picking/route level.</t>
         </is>
@@ -2867,7 +3003,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr"/>
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>Default days to ship. Odoo manages on products/routes.</t>
         </is>
@@ -2896,7 +3033,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>many2one → delivery.carrier</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2905,6 +3042,11 @@
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>delivery.carrier</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>Default shipping method. Requires delivery carriers to be configured.</t>
         </is>
@@ -2941,7 +3083,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>Default days to receive purchases. Odoo uses product supplierinfo.</t>
         </is>
@@ -2978,7 +3121,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr"/>
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>Drop-ship capability. Odoo handles via routes.</t>
         </is>
@@ -3015,7 +3159,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G68" s="2" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>Default GL for purchase costs. Odoo has no per-partner purchase GL offset.</t>
         </is>
@@ -3052,7 +3197,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>Default GL for sales revenue. Odoo has no per-partner sales GL offset.</t>
         </is>
@@ -3081,7 +3227,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>many2one → account.account</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -3090,6 +3236,11 @@
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>account.account</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>Default Accounts Payable GL. Resolve via account.account lookup.</t>
         </is>
@@ -3118,7 +3269,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>many2one → account.account</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -3127,6 +3278,11 @@
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>account.account</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t>Default Accounts Receivable GL. Resolve via account.account lookup.</t>
         </is>
@@ -3163,7 +3319,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G72" s="2" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>Tax identification number. Odoo validates per country.</t>
         </is>
@@ -3200,7 +3357,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G73" s="2" t="inlineStr">
+      <c r="G73" s="2" t="inlineStr"/>
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t>Chamber of commerce / company registration number.</t>
         </is>
@@ -3237,7 +3395,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr">
+      <c r="G74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr">
         <is>
           <t>Dutch Citizen Service Number. Sensitive PII.</t>
         </is>
@@ -3274,7 +3433,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr">
+      <c r="G75" s="2" t="inlineStr"/>
+      <c r="H75" s="2" t="inlineStr">
         <is>
           <t>Dutch fiscal number.</t>
         </is>
@@ -3311,7 +3471,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr">
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr">
         <is>
           <t>Dutch government ID number.</t>
         </is>
@@ -3348,7 +3509,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr">
+      <c r="G77" s="2" t="inlineStr"/>
+      <c r="H77" s="2" t="inlineStr">
         <is>
           <t>Global Location Number.</t>
         </is>
@@ -3385,7 +3547,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr">
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr">
         <is>
           <t>EU customs EORI number.</t>
         </is>
@@ -3422,7 +3585,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G79" s="2" t="inlineStr">
+      <c r="G79" s="2" t="inlineStr"/>
+      <c r="H79" s="2" t="inlineStr">
         <is>
           <t>VAT status for Belgian listing.</t>
         </is>
@@ -3459,7 +3623,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G80" s="2" t="inlineStr">
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr">
         <is>
           <t>Withholding tax on sales.</t>
         </is>
@@ -3496,7 +3661,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G81" s="2" t="inlineStr">
+      <c r="G81" s="2" t="inlineStr"/>
+      <c r="H81" s="2" t="inlineStr">
         <is>
           <t>Belgian Belcotax relation.</t>
         </is>
@@ -3533,7 +3699,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G82" s="2" t="inlineStr">
+      <c r="G82" s="2" t="inlineStr"/>
+      <c r="H82" s="2" t="inlineStr">
         <is>
           <t>UK loan repayment plan.</t>
         </is>
@@ -3570,7 +3737,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr">
+      <c r="G83" s="2" t="inlineStr"/>
+      <c r="H83" s="2" t="inlineStr">
         <is>
           <t>UK unique taxpayer reference.</t>
         </is>
@@ -3607,7 +3775,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G84" s="2" t="inlineStr">
+      <c r="G84" s="2" t="inlineStr"/>
+      <c r="H84" s="2" t="inlineStr">
         <is>
           <t>DATEV creditor code (German).</t>
         </is>
@@ -3644,7 +3813,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G85" s="2" t="inlineStr">
+      <c r="G85" s="2" t="inlineStr"/>
+      <c r="H85" s="2" t="inlineStr">
         <is>
           <t>DATEV debtor code (German).</t>
         </is>
@@ -3681,7 +3851,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G86" s="2" t="inlineStr">
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr">
         <is>
           <t>Suppress DATEV duplicate warnings.</t>
         </is>
@@ -3718,7 +3889,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G87" s="2" t="inlineStr">
+      <c r="G87" s="2" t="inlineStr"/>
+      <c r="H87" s="2" t="inlineStr">
         <is>
           <t>Peppol endpoint identifier. Direct semantic match.</t>
         </is>
@@ -3755,7 +3927,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G88" s="2" t="inlineStr">
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr">
         <is>
           <t>Peppol identifier type (numeric). Odoo has peppol_eas (selection with EAS codes). Value sets may not align.</t>
         </is>
@@ -3792,7 +3965,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G89" s="2" t="inlineStr">
+      <c r="G89" s="2" t="inlineStr"/>
+      <c r="H89" s="2" t="inlineStr">
         <is>
           <t>Incoterm code for purchases. Odoo manages at order level.</t>
         </is>
@@ -3829,7 +4003,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G90" s="2" t="inlineStr">
+      <c r="G90" s="2" t="inlineStr"/>
+      <c r="H90" s="2" t="inlineStr">
         <is>
           <t>Incoterm code for sales.</t>
         </is>
@@ -3866,7 +4041,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G91" s="2" t="inlineStr">
+      <c r="G91" s="2" t="inlineStr"/>
+      <c r="H91" s="2" t="inlineStr">
         <is>
           <t>Incoterm location for purchases.</t>
         </is>
@@ -3903,7 +4079,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G92" s="2" t="inlineStr">
+      <c r="G92" s="2" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr">
         <is>
           <t>Incoterm location for sales.</t>
         </is>
@@ -3940,7 +4117,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G93" s="2" t="inlineStr">
+      <c r="G93" s="2" t="inlineStr"/>
+      <c r="H93" s="2" t="inlineStr">
         <is>
           <t>Incoterm version for purchases (2010/2020).</t>
         </is>
@@ -3977,7 +4155,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G94" s="2" t="inlineStr">
+      <c r="G94" s="2" t="inlineStr"/>
+      <c r="H94" s="2" t="inlineStr">
         <is>
           <t>Incoterm version for sales (2010/2020).</t>
         </is>
@@ -4014,7 +4193,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G95" s="2" t="inlineStr">
+      <c r="G95" s="2" t="inlineStr"/>
+      <c r="H95" s="2" t="inlineStr">
         <is>
           <t>Intrastat area. Odoo manages at invoice line level.</t>
         </is>
@@ -4051,7 +4231,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G96" s="2" t="inlineStr">
+      <c r="G96" s="2" t="inlineStr"/>
+      <c r="H96" s="2" t="inlineStr">
         <is>
           <t>Intrastat delivery method.</t>
         </is>
@@ -4088,7 +4269,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G97" s="2" t="inlineStr">
+      <c r="G97" s="2" t="inlineStr"/>
+      <c r="H97" s="2" t="inlineStr">
         <is>
           <t>Intrastat system code.</t>
         </is>
@@ -4125,7 +4307,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G98" s="2" t="inlineStr">
+      <c r="G98" s="2" t="inlineStr"/>
+      <c r="H98" s="2" t="inlineStr">
         <is>
           <t>Intrastat transaction type A.</t>
         </is>
@@ -4162,7 +4345,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G99" s="2" t="inlineStr">
+      <c r="G99" s="2" t="inlineStr"/>
+      <c r="H99" s="2" t="inlineStr">
         <is>
           <t>Intrastat transaction type B.</t>
         </is>
@@ -4199,7 +4383,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G100" s="2" t="inlineStr">
+      <c r="G100" s="2" t="inlineStr"/>
+      <c r="H100" s="2" t="inlineStr">
         <is>
           <t>Intrastat transport method.</t>
         </is>
@@ -4228,7 +4413,7 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.users</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -4237,6 +4422,11 @@
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>res.users</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
         <is>
           <t>Account manager → Odoo salesperson.</t>
         </is>
@@ -4275,6 +4465,11 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -4312,6 +4507,11 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
           <t>Redundant numeric ID.</t>
         </is>
       </c>
@@ -4347,7 +4547,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G104" s="2" t="inlineStr">
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr">
         <is>
           <t>Reference to accountant (another Account). Store GUID.</t>
         </is>
@@ -4376,7 +4577,7 @@
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.partner</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
@@ -4385,6 +4586,11 @@
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>res.partner</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
         <is>
           <t>Parent account (self-referential hierarchy). Resolve via x_aa_exact_account_id lookup. Ensure parent accounts migrated before children.</t>
         </is>
@@ -4421,7 +4627,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G106" s="2" t="inlineStr">
+      <c r="G106" s="2" t="inlineStr"/>
+      <c r="H106" s="2" t="inlineStr">
         <is>
           <t>Main contact person GUID. After Contact migration, can be cross-referenced via x_aa_exact_contact_id on the child partner.</t>
         </is>
@@ -4458,7 +4665,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G107" s="2" t="inlineStr">
+      <c r="G107" s="2" t="inlineStr"/>
+      <c r="H107" s="2" t="inlineStr">
         <is>
           <t>Reference to reseller account. Store GUID.</t>
         </is>
@@ -4497,6 +4705,11 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -4534,6 +4747,11 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -4561,7 +4779,7 @@
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.partner.industry</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -4570,6 +4788,11 @@
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>res.partner.industry</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
         <is>
           <t>Activity sector → Odoo industry. Not core to subscriptions — resolve later if needed.</t>
         </is>
@@ -4606,7 +4829,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G111" s="2" t="inlineStr">
+      <c r="G111" s="2" t="inlineStr"/>
+      <c r="H111" s="2" t="inlineStr">
         <is>
           <t>Sub-sector. No Odoo sub-industry. Store GUID.</t>
         </is>
@@ -4643,7 +4867,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G112" s="2" t="inlineStr">
+      <c r="G112" s="2" t="inlineStr"/>
+      <c r="H112" s="2" t="inlineStr">
         <is>
           <t>Lead purpose GUID. Shared field name with Contacts sheet.</t>
         </is>
@@ -4680,7 +4905,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G113" s="2" t="inlineStr">
+      <c r="G113" s="2" t="inlineStr"/>
+      <c r="H113" s="2" t="inlineStr">
         <is>
           <t>Lead source GUID. Shared field name with Contacts sheet.</t>
         </is>
@@ -4717,7 +4943,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G114" s="2" t="inlineStr">
+      <c r="G114" s="2" t="inlineStr"/>
+      <c r="H114" s="2" t="inlineStr">
         <is>
           <t>Business type GUID.</t>
         </is>
@@ -4754,7 +4981,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G115" s="2" t="inlineStr">
+      <c r="G115" s="2" t="inlineStr"/>
+      <c r="H115" s="2" t="inlineStr">
         <is>
           <t>Company size GUID.</t>
         </is>
@@ -4791,7 +5019,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G116" s="2" t="inlineStr">
+      <c r="G116" s="2" t="inlineStr"/>
+      <c r="H116" s="2" t="inlineStr">
         <is>
           <t>Code under which your company is known at this account.</t>
         </is>
@@ -4828,7 +5057,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G117" s="2" t="inlineStr">
+      <c r="G117" s="2" t="inlineStr"/>
+      <c r="H117" s="2" t="inlineStr">
         <is>
           <t>Account classification 1 (of 8). Store GUID.</t>
         </is>
@@ -4865,7 +5095,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G118" s="2" t="inlineStr">
+      <c r="G118" s="2" t="inlineStr"/>
+      <c r="H118" s="2" t="inlineStr">
         <is>
           <t>Account classification 2. Store GUID.</t>
         </is>
@@ -4902,7 +5133,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G119" s="2" t="inlineStr">
+      <c r="G119" s="2" t="inlineStr"/>
+      <c r="H119" s="2" t="inlineStr">
         <is>
           <t>Account classification 3. Store GUID.</t>
         </is>
@@ -4939,7 +5171,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G120" s="2" t="inlineStr">
+      <c r="G120" s="2" t="inlineStr"/>
+      <c r="H120" s="2" t="inlineStr">
         <is>
           <t>Account classification 4. Store GUID.</t>
         </is>
@@ -4976,7 +5209,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G121" s="2" t="inlineStr">
+      <c r="G121" s="2" t="inlineStr"/>
+      <c r="H121" s="2" t="inlineStr">
         <is>
           <t>Account classification 5. Store GUID.</t>
         </is>
@@ -5013,7 +5247,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G122" s="2" t="inlineStr">
+      <c r="G122" s="2" t="inlineStr"/>
+      <c r="H122" s="2" t="inlineStr">
         <is>
           <t>Account classification 6. Store GUID.</t>
         </is>
@@ -5050,7 +5285,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G123" s="2" t="inlineStr">
+      <c r="G123" s="2" t="inlineStr"/>
+      <c r="H123" s="2" t="inlineStr">
         <is>
           <t>Account classification 7. Store GUID.</t>
         </is>
@@ -5087,7 +5323,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G124" s="2" t="inlineStr">
+      <c r="G124" s="2" t="inlineStr"/>
+      <c r="H124" s="2" t="inlineStr">
         <is>
           <t>Account classification 8. Store GUID.</t>
         </is>
@@ -5124,7 +5361,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G125" s="2" t="inlineStr">
+      <c r="G125" s="2" t="inlineStr"/>
+      <c r="H125" s="2" t="inlineStr">
         <is>
           <t>Account start date. Shared field name with Contacts sheet. Strip time.</t>
         </is>
@@ -5161,7 +5399,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G126" s="2" t="inlineStr">
+      <c r="G126" s="2" t="inlineStr"/>
+      <c r="H126" s="2" t="inlineStr">
         <is>
           <t>Account end date. Used in Derived: active. Shared field name with Contacts sheet.</t>
         </is>
@@ -5198,7 +5437,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G127" s="2" t="inlineStr">
+      <c r="G127" s="2" t="inlineStr"/>
+      <c r="H127" s="2" t="inlineStr">
         <is>
           <t>Company registration date. Strip time.</t>
         </is>
@@ -5235,7 +5475,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G128" s="2" t="inlineStr">
+      <c r="G128" s="2" t="inlineStr"/>
+      <c r="H128" s="2" t="inlineStr">
         <is>
           <t>Date of latest external data verification.</t>
         </is>
@@ -5272,7 +5513,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G129" s="2" t="inlineStr">
+      <c r="G129" s="2" t="inlineStr"/>
+      <c r="H129" s="2" t="inlineStr">
         <is>
           <t>Company logo. Odoo auto-generates smaller sizes.</t>
         </is>
@@ -5309,7 +5551,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G130" s="2" t="inlineStr">
+      <c r="G130" s="2" t="inlineStr"/>
+      <c r="H130" s="2" t="inlineStr">
         <is>
           <t>Original filename. Odoo does not store filenames.</t>
         </is>
@@ -5348,6 +5591,11 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
           <t>Exact-hosted URL. Not meaningful post-migration.</t>
         </is>
       </c>
@@ -5385,6 +5633,11 @@
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
           <t>Exact-hosted URL. Not meaningful post-migration.</t>
         </is>
       </c>
@@ -5420,7 +5673,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G133" s="2" t="inlineStr">
+      <c r="G133" s="2" t="inlineStr"/>
+      <c r="H133" s="2" t="inlineStr">
         <is>
           <t>Language code. Exact ISO → Odoo locale (e.g., "NL" → "nl_NL"). Same logic as Contacts sheet.</t>
         </is>
@@ -5459,6 +5713,11 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -5494,7 +5753,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G135" s="2" t="inlineStr">
+      <c r="G135" s="2" t="inlineStr"/>
+      <c r="H135" s="2" t="inlineStr">
         <is>
           <t>Account remarks. Wrap in &lt;p&gt; tags. Same target as Contacts (Notes → comment).</t>
         </is>
@@ -5533,6 +5793,11 @@
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
           <t>Bank accounts collection. Deferred to later batch → res.partner.bank.</t>
         </is>
       </c>
@@ -5568,7 +5833,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G137" s="2" t="inlineStr">
+      <c r="G137" s="2" t="inlineStr"/>
+      <c r="H137" s="2" t="inlineStr">
         <is>
           <t>Blocked flag. May feed into Derived: active logic.</t>
         </is>
@@ -5605,7 +5871,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G138" s="2" t="inlineStr">
+      <c r="G138" s="2" t="inlineStr"/>
+      <c r="H138" s="2" t="inlineStr">
         <is>
           <t>Security level (0-100).</t>
         </is>
@@ -5642,7 +5909,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G139" s="2" t="inlineStr">
+      <c r="G139" s="2" t="inlineStr"/>
+      <c r="H139" s="2" t="inlineStr">
         <is>
           <t>CRM creation source.</t>
         </is>
@@ -5679,7 +5947,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G140" s="2" t="inlineStr">
+      <c r="G140" s="2" t="inlineStr"/>
+      <c r="H140" s="2" t="inlineStr">
         <is>
           <t>Auto-create entries for complete proposals.</t>
         </is>
@@ -5716,7 +5985,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G141" s="2" t="inlineStr">
+      <c r="G141" s="2" t="inlineStr"/>
+      <c r="H141" s="2" t="inlineStr">
         <is>
           <t>Creation timestamp.</t>
         </is>
@@ -5745,7 +6015,7 @@
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.users</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
@@ -5754,6 +6024,11 @@
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>res.users</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
         <is>
           <t>Creator. Resolve via res.users. Default to admin.</t>
         </is>
@@ -5792,6 +6067,11 @@
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -5827,7 +6107,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G144" s="2" t="inlineStr">
+      <c r="G144" s="2" t="inlineStr"/>
+      <c r="H144" s="2" t="inlineStr">
         <is>
           <t>Last modification timestamp.</t>
         </is>
@@ -5856,7 +6137,7 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.users</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
@@ -5865,6 +6146,11 @@
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>res.users</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
         <is>
           <t>Modifier. Resolve via res.users. Default to admin.</t>
         </is>
@@ -5903,6 +6189,11 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -5930,7 +6221,7 @@
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.company</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
@@ -5939,6 +6230,11 @@
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>res.company</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
         <is>
           <t>Exact division → res.company.</t>
         </is>
@@ -5977,6 +6273,11 @@
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6014,6 +6315,11 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6051,6 +6357,11 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6088,6 +6399,11 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
           <t>Obsolete. Use SalesCurrency / PurchaseCurrency.</t>
         </is>
       </c>
@@ -6125,6 +6441,11 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6162,6 +6483,11 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6199,6 +6525,11 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6236,6 +6567,11 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6273,6 +6609,11 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6310,6 +6651,11 @@
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6347,6 +6693,11 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6384,6 +6735,11 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6421,6 +6777,11 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6458,6 +6819,11 @@
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6495,6 +6861,11 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6532,6 +6903,11 @@
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6569,6 +6945,11 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -6606,6 +6987,11 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
           <t>Premium endpoint reference. Always skip.</t>
         </is>
       </c>
@@ -6641,7 +7027,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G166" s="2" t="inlineStr">
+      <c r="G166" s="2" t="inlineStr"/>
+      <c r="H166" s="2" t="inlineStr">
         <is>
           <t>Always True for Accounts. (Contacts sheet sets False.)</t>
         </is>
@@ -6678,7 +7065,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G167" s="2" t="inlineStr">
+      <c r="G167" s="2" t="inlineStr"/>
+      <c r="H167" s="2" t="inlineStr">
         <is>
           <t>Always "company". (Contacts sheet sets "person".)</t>
         </is>
@@ -6715,7 +7103,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G168" s="2" t="inlineStr">
+      <c r="G168" s="2" t="inlineStr"/>
+      <c r="H168" s="2" t="inlineStr">
         <is>
           <t>Set to 1 if Status="C", else 0. Contacts inherit from parent — do not set on person records.</t>
         </is>
@@ -6752,7 +7141,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G169" s="2" t="inlineStr">
+      <c r="G169" s="2" t="inlineStr"/>
+      <c r="H169" s="2" t="inlineStr">
         <is>
           <t>Set to 1 if IsSupplier=True, else 0. Contacts inherit from parent.</t>
         </is>
@@ -6789,7 +7179,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G170" s="2" t="inlineStr">
+      <c r="G170" s="2" t="inlineStr"/>
+      <c r="H170" s="2" t="inlineStr">
         <is>
           <t>False if EndDate &lt; migration date, else True. Optionally also False if Blocked=True.</t>
         </is>
@@ -6826,7 +7217,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G171" s="2" t="inlineStr">
+      <c r="G171" s="2" t="inlineStr"/>
+      <c r="H171" s="2" t="inlineStr">
         <is>
           <t>True if CreditLineSales &gt; 0. Required for Odoo to enforce credit_limit.</t>
         </is>
@@ -6863,14 +7255,15 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G172" s="2" t="inlineStr">
+      <c r="G172" s="2" t="inlineStr"/>
+      <c r="H172" s="2" t="inlineStr">
         <is>
           <t>Set to "contact" (default address type for company-level partners).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6881,7 +7274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -6890,7 +7283,8 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="12.5" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6926,6 +7320,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Related Model</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -6961,7 +7360,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Primary key. Named x_aa_exact_contact_id to distinguish from x_aa_exact_account_id (Accounts sheet). A person partner has this field populated; a company partner does not.</t>
         </is>
@@ -6998,7 +7398,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Numeric contact ID in Exact.</t>
         </is>
@@ -7035,7 +7436,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Code of the parent account (denormalized). The authoritative account code is on the parent partner's ref field.</t>
         </is>
@@ -7064,7 +7466,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.partner</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -7073,6 +7475,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>res.partner</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>The account this contact belongs to. Resolve via x_aa_exact_account_id lookup on company partners. PREREQUISITE: Accounts must be migrated first.</t>
         </is>
@@ -7111,6 +7518,11 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
           <t>Denormalized. Derivable from parent_id.name.</t>
         </is>
       </c>
@@ -7148,6 +7560,11 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
           <t>Denormalized. Already on parent partner via customer_rank.</t>
         </is>
       </c>
@@ -7185,6 +7602,11 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
           <t>Denormalized. Already on parent partner via supplier_rank.</t>
         </is>
       </c>
@@ -7222,6 +7644,11 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
           <t>Account-level concept. Already on parent partner as x_aa_main_contact_id.</t>
         </is>
       </c>
@@ -7257,7 +7684,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>First name. Preserved to retain name parts. Also used to derive name (see Derived).</t>
         </is>
@@ -7294,7 +7722,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Middle name / tussenvoegsel.</t>
         </is>
@@ -7331,7 +7760,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Last name. Also used to derive name.</t>
         </is>
@@ -7368,7 +7798,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Initials.</t>
         </is>
@@ -7407,6 +7838,11 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
           <t>Denormalized composite. We derive name from the individual parts instead.</t>
         </is>
       </c>
@@ -7442,7 +7878,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Last name of spouse/partner.</t>
         </is>
@@ -7479,7 +7916,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Middle name of spouse/partner.</t>
         </is>
@@ -7516,7 +7954,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Title code (e.g., Mr, Mrs). Odoo has title (many2one → res.partner.title) but code sets may differ. Preserve raw; optionally resolve to res.partner.title.</t>
         </is>
@@ -7553,7 +7992,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Title abbreviation.</t>
         </is>
@@ -7590,7 +8030,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Title description. Could map to res.partner.title.name if a clean mapping exists.</t>
         </is>
@@ -7627,7 +8068,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Job title → Odoo function. Direct match.</t>
         </is>
@@ -7664,7 +8106,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Gender code.</t>
         </is>
@@ -7701,7 +8144,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Date of birth. Strip time.</t>
         </is>
@@ -7738,7 +8182,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Place of birth.</t>
         </is>
@@ -7775,7 +8220,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Nationality code.</t>
         </is>
@@ -7812,7 +8258,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>SSN. Sensitive PII.</t>
         </is>
@@ -7849,7 +8296,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Reference to Exact personal information entity. Store GUID.</t>
         </is>
@@ -7886,7 +8334,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Identity verification date. Strip time.</t>
         </is>
@@ -7923,7 +8372,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Identification document GUID.</t>
         </is>
@@ -7960,7 +8410,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>User who performed identification. Store GUID.</t>
         </is>
@@ -7997,7 +8448,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Street name. Concatenate: "{AddressStreet} {AddressStreetNumber}{AddressStreetNumberSuffix}" → street. Only set if contact has own address; otherwise leave empty so Odoo inherits from parent_id.</t>
         </is>
@@ -8034,7 +8486,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Street number. Preserved for fidelity. Used in street concatenation.</t>
         </is>
@@ -8071,7 +8524,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Street number suffix. Used in street concatenation.</t>
         </is>
@@ -8108,7 +8562,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Second address line. Only set if contact has own address.</t>
         </is>
@@ -8145,7 +8600,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Only set if contact has own address.</t>
         </is>
@@ -8182,7 +8638,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Only set if contact has own address.</t>
         </is>
@@ -8211,7 +8668,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.country</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -8220,6 +8677,11 @@
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>res.country</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Country code → res.country.code lookup. Only set if contact has own address.</t>
         </is>
@@ -8248,7 +8710,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.country.state</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -8257,6 +8719,11 @@
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>res.country.state</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>State/Province code. Only set if contact has own address.</t>
         </is>
@@ -8293,7 +8760,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Business email → Odoo email (primary). If empty, fall back to Email field.</t>
         </is>
@@ -8330,7 +8798,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Personal/secondary email. Used as fallback for Odoo email if BusinessEmail is empty.</t>
         </is>
@@ -8367,7 +8836,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Business phone → Odoo phone.</t>
         </is>
@@ -8404,7 +8874,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Phone extension. Shared field name with Accounts sheet.</t>
         </is>
@@ -8441,7 +8912,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Fax. Shared field name with Accounts sheet.</t>
         </is>
@@ -8478,7 +8950,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Business mobile → Odoo mobile. If empty, fall back to Mobile field.</t>
         </is>
@@ -8515,7 +8988,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Personal phone.</t>
         </is>
@@ -8552,7 +9026,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Personal phone extension.</t>
         </is>
@@ -8589,7 +9064,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>Personal mobile. Used as fallback for Odoo mobile if BusinessMobile is empty.</t>
         </is>
@@ -8626,7 +9102,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Main contact flag. Cross-ref: parent account has x_aa_main_contact_id storing this contact's GUID.</t>
         </is>
@@ -8663,7 +9140,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>Lead purpose GUID. Shared field name with Accounts sheet.</t>
         </is>
@@ -8700,7 +9178,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Lead source GUID. Shared field name with Accounts sheet.</t>
         </is>
@@ -8737,7 +9216,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>Free-text marketing notes.</t>
         </is>
@@ -8774,7 +9254,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Excluded from mailings. Consider also setting is_blacklisted=True.</t>
         </is>
@@ -8811,7 +9292,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>Remarks/notes. Wrap in &lt;p&gt; tags. Same target field as Accounts (Remarks → comment).</t>
         </is>
@@ -8848,7 +9330,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>Contact start date. Shared field name with Accounts sheet. Strip time.</t>
         </is>
@@ -8885,7 +9368,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>Contact end date. Used in Derived: active. Shared field name with Accounts sheet.</t>
         </is>
@@ -8922,7 +9406,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>Contact photo. Write-only in Exact; fetch via PictureUrl during extraction.</t>
         </is>
@@ -8959,7 +9444,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>Original filename.</t>
         </is>
@@ -8998,6 +9484,11 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
           <t>Exact-hosted URL. Not meaningful post-migration.</t>
         </is>
       </c>
@@ -9035,6 +9526,11 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
           <t>Exact-hosted URL. Used during extraction only.</t>
         </is>
       </c>
@@ -9070,7 +9566,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>Language code. Same ISO → locale logic as Accounts sheet.</t>
         </is>
@@ -9107,7 +9604,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>Anonymisation flag. Shared field name with Accounts sheet.</t>
         </is>
@@ -9144,7 +9642,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>Creation timestamp.</t>
         </is>
@@ -9173,7 +9672,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.users</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -9182,6 +9681,11 @@
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>res.users</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>Creator. Default to admin if not mapped.</t>
         </is>
@@ -9220,6 +9724,11 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -9255,7 +9764,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr"/>
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>Last modification timestamp.</t>
         </is>
@@ -9284,7 +9794,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.users</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -9293,6 +9803,11 @@
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>res.users</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>Modifier. Default to admin.</t>
         </is>
@@ -9331,6 +9846,11 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -9358,7 +9878,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.company</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -9367,6 +9887,11 @@
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>res.company</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>Exact division → res.company.</t>
         </is>
@@ -9405,6 +9930,11 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
           <t>Obsolete.</t>
         </is>
       </c>
@@ -9442,6 +9972,11 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
           <t>Obsolete. May overwrite LastName.</t>
         </is>
       </c>
@@ -9479,6 +10014,11 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
           <t>Obsolete. May overwrite MiddleName.</t>
         </is>
       </c>
@@ -9516,6 +10056,11 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
           <t>Premium endpoint reference. Always skip.</t>
         </is>
       </c>
@@ -9551,7 +10096,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G72" s="2" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>Always False for Contacts. (Accounts sheet sets True.)</t>
         </is>
@@ -9588,7 +10134,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G73" s="2" t="inlineStr">
+      <c r="G73" s="2" t="inlineStr"/>
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t>Always "person". (Accounts sheet sets "company".)</t>
         </is>
@@ -9625,7 +10172,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr">
+      <c r="G74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr">
         <is>
           <t>Concatenated: "{FirstName} {MiddleName} {LastName}".strip(), skipping empty parts. Fall back to FullName if both FirstName and LastName are empty.</t>
         </is>
@@ -9662,7 +10210,8 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr">
+      <c r="G75" s="2" t="inlineStr"/>
+      <c r="H75" s="2" t="inlineStr">
         <is>
           <t>False if EndDate &lt; migration date, else True. Same logic as Accounts sheet.</t>
         </is>
@@ -9699,14 +10248,15 @@
           <t>res.partner</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr">
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr">
         <is>
           <t>Set to "contact" (default address type for person contacts).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9717,7 +10267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -9726,7 +10276,8 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="12.5" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9762,6 +10313,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Related Model</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -9797,7 +10353,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Primary key. Stored for reconciliation, re-runs, and relationship resolution from Accounts and Subscriptions.</t>
         </is>
@@ -9834,7 +10391,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Exact payment condition code. Odoo has no code field on payment terms — identification is by name and ID. This code is the lookup key used in Exact Accounts (PaymentConditionSales, PaymentConditionPurchase), so it must be stored for resolution.</t>
         </is>
@@ -9871,7 +10429,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Description of the payment condition → Odoo payment term name.</t>
         </is>
@@ -9908,7 +10467,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Number of days added to due date calculation. Preserved on header for reference. Also used to derive the account.payment.term.line record (see child sheet). Note: the combination of PaymentEndOfMonths + PaymentDays defines the full due date logic.</t>
         </is>
@@ -9945,7 +10505,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Number of month-end periods before adding PaymentDays. Preserved on header. Used to derive delay_type on the child line. Mapping: 0 → "days_after_invoice_date", 1 → "days_after_end_of_month", 2+ → "days_after_end_of_month" with adjusted nb_days (approximate — Odoo has no native multi-month-end concept; complex cases may need manual review).</t>
         </is>
@@ -9982,7 +10543,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Fraction of total invoice amount for this condition (e.g., 1.0 = 100%). Preserved on header. Used to derive child line value/value_amount. If 1.0 or null → line value="balance"; if &lt; 1.0 → line value="percent", value_amount = Percentage * 100.</t>
         </is>
@@ -10019,7 +10581,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Method of payment (B=On credit, I=Collection, K=Cash, Q=PSP Collection). No Odoo equivalent on payment terms — Odoo handles payment methods on journals and payment records, not on terms. Preserve as custom.</t>
         </is>
@@ -10056,7 +10619,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Early payment discount percentage. Direct mapping. Exact stores as fraction (e.g., 0.02); Odoo stores as percentage (e.g., 2.0). Convert: multiply by 100 during migration. Also set early_discount=True if value &gt; 0 (see Derived rows).</t>
         </is>
@@ -10093,7 +10657,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Number of days to pay early to qualify for discount. Direct mapping.</t>
         </is>
@@ -10130,7 +10695,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>How discount is calculated relative to VAT (E=Excluding VAT, I=Including VAT). Preserved as custom. Also used in combination with VATCalculation to derive early_pay_discount_computation (see Derived rows).</t>
         </is>
@@ -10167,7 +10733,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>How VAT is calculated relative to discount (E=Excluding discount, I=Including discount). Preserved as custom. Used jointly with DiscountCalculation to derive early_pay_discount_computation.</t>
         </is>
@@ -10204,7 +10771,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Type of discount: B=Settlement discount, K=Credit surcharge. No Odoo equivalent. Preserve as custom.</t>
         </is>
@@ -10241,7 +10809,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Default credit management scenario GUID. No Odoo equivalent on payment terms. Preserve GUID.</t>
         </is>
@@ -10280,6 +10849,11 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field for CreditManagementScenario.</t>
         </is>
       </c>
@@ -10317,6 +10891,11 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field for CreditManagementScenario.</t>
         </is>
       </c>
@@ -10352,7 +10931,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Creation timestamp. Direct mapping.</t>
         </is>
@@ -10381,7 +10961,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.users</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -10390,6 +10970,11 @@
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>res.users</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Creator user GUID. Resolve via res.users lookup. Default to admin if not mapped.</t>
         </is>
@@ -10428,6 +11013,11 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -10463,7 +11053,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Last modification timestamp. Direct mapping.</t>
         </is>
@@ -10492,7 +11083,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.users</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -10501,6 +11092,11 @@
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>res.users</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Modifier user GUID. Resolve via res.users lookup. Default to admin if not mapped.</t>
         </is>
@@ -10539,6 +11135,11 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
           <t>Denormalized display field.</t>
         </is>
       </c>
@@ -10566,7 +11167,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>many2one → res.company</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -10575,6 +11176,11 @@
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>res.company</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Exact division code. Resolve to res.company. For single-company setups, hardcode.</t>
         </is>
@@ -10611,7 +11217,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Set to True if DiscountPercentage &gt; 0, else False. Enables the early discount UI and computation in Odoo.</t>
         </is>
@@ -10648,7 +11255,8 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Derived from DiscountCalculation + VATCalculation combination. Mapping: if VATCalculation="E" (VAT excludes discount) → "excluded" (tax never reduced); if VATCalculation="I" and DiscountCalculation="I" → "always" (tax always reduced based on discounted amount); if VATCalculation="I" and DiscountCalculation="E" → "mixed" (tax reduced only when discount actually taken). Default to "excluded" if no discount. Review with accounting team — this mapping is approximate and business-critical.</t>
         </is>
@@ -10685,14 +11293,15 @@
           <t>account.payment.term</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Set to True for all migrated payment terms. Deactivate manually post-migration if any are no longer in use.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10703,7 +11312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -10712,7 +11321,8 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="12.5" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10748,6 +11358,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Related Model</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -10775,7 +11390,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>many2one → account.payment.term</t>
+          <t>many2one</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -10784,6 +11399,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>account.payment.term</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Reference to the parent account.payment.term record created from the same Exact PaymentCondition. Set during migration via the parent record's ID.</t>
         </is>
@@ -10820,7 +11440,8 @@
           <t>account.payment.term.line</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Derived from Exact Percentage field. If Percentage is null, empty, or 1.0 → "balance" (full remaining amount). If Percentage &lt; 1.0 → "percent". Most Exact payment conditions use a single 100% term, so "balance" will be the common case.</t>
         </is>
@@ -10857,7 +11478,8 @@
           <t>account.payment.term.line</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Derived from Exact Percentage field. If value="balance" → 0.0 (Odoo ignores this for balance lines). If value="percent" → Percentage * 100 (e.g., 0.5 → 50.0). Exact stores as fraction; Odoo stores as percentage.</t>
         </is>
@@ -10894,7 +11516,8 @@
           <t>account.payment.term.line</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Derived from Exact PaymentEndOfMonths. Mapping: PaymentEndOfMonths=0 → "days_after_invoice_date" (simple net days); PaymentEndOfMonths=1 → "days_after_end_of_month" (end of invoice month + PaymentDays); PaymentEndOfMonths≥2 → "days_after_end_of_month" with nb_days adjusted to approximate (e.g., EndOfMonths=2, PaymentDays=15 → nb_days=15 with a note that this is approximate). Complex multi-month-end cases should be flagged for manual review.</t>
         </is>
@@ -10931,7 +11554,8 @@
           <t>account.payment.term.line</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Derived from Exact PaymentDays (and PaymentEndOfMonths for adjustments). For simple cases: nb_days = PaymentDays. For PaymentEndOfMonths≥2: nb_days = PaymentDays + ((PaymentEndOfMonths - 1) * 30) as an approximation, flagged for review.</t>
         </is>
@@ -10968,14 +11592,15 @@
           <t>account.payment.term.line</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Set to "0" (default). Only relevant when delay_type involves end-of-month calculations and a buffer is needed. Can be adjusted manually post-migration for edge cases.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
updated skills to always mark pk's as Direct mapping
</commit_message>
<xml_diff>
--- a/mappings/contacts_mapping.xlsx
+++ b/mappings/contacts_mapping.xlsx
@@ -7,17 +7,17 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts → res.partner" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts → res.partner" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PaymentCond → payment.term" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PaymentCond → payment.term.line" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRMAccounts → res.partner" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRMContacts → res.partner" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CashflowPaym... → account..." sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CashflowPaym... → account...1" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Accounts → res.partner'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Contacts → res.partner'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'PaymentCond → payment.term'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PaymentCond → payment.term.line'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CRMAccounts → res.partner'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CRMContacts → res.partner'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CashflowPaym... → account...'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CashflowPaym... → account...1'!$A$1:$H$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>

</xml_diff>